<commit_message>
Build V1 real-data pipeline, output pack, and tracker-style HTML dashboard
- Fund investment deep-dive: New Space GP Com SCSp, MGX GP/HoldCo, MGX Denali valuation added with primary-document citations
- Fixed valuation rollup bug (sub-vehicle carrying values were being collapsed instead of summed)
- Fixed 3 silently-unresolved tracker-only entities (X-fusion, Jollychic, Honor Device Co Ltd)
- Added generate-output-pack CLI command (full V1 Output Pack workbook + Markdown summary note)
- Added generate-tracker-dashboard CLI command: HTML dashboard mirroring the tracker's own Live/Exited report structure (sectioned by Investing Entity), with deal- and section-level IRR, hover tooltips citing data provenance, CSV export, full cashflow/ownership/change-log tabs, historical NAV + quarterly cashflow charts
- Added scan-for-updates CLI command (real folder-diff scan for new/changed investments)
- Updated PRD changelog and V1 Input Data Spec to reflect all adapters built this session
</commit_message>
<xml_diff>
--- a/data/outputs/Investment_Register_Intake.xlsx
+++ b/data/outputs/Investment_Register_Intake.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment_Register_Draft" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Document_Extract" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Needs_Source_Documents" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,488 +481,2032 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AppliedAI-CONV-2022</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AAICO (desktop)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+          <t>Applied AI</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mozn Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Convertible</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2022-09-01</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\AAICO (desktop)\2. Transaction Closure\ADIO - Applied AI Co. Ltd. - Non Binding Term Sheet - 19 Aug 2022 - Signed (002).pdf</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
+          <t>...\AAICO (desktop)\2. Transaction Closure\3. Transaction Final Docs (Aug 22)\Final docs - 09 Sep\220908 - G42 Convertible Note EXECUTED ^^^.pdf</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>CONFIRMED from executed Convertible Note (220908 - G42 Convertible Note EXECUTED): Purchase Price $15,000,000, Funding Date 1 Sep 2022, Company: Applied AI Corporation Limited (ADGM), Investor: Mozn Holding RSC Ltd. Guaranteed by Applied AI Corporation Limited (UK entity, Co. No. 13263710). Note funded via multiple 'Tranche Funding Dates' per an associated Process Letter - consistent with tracker showing 4 actual draws (2022-10-27 $4.75M, 2023-07-14 $2.75M, 2024-01-04 $4.0M, 2024-11-21 $3.5M = $15M). This Note is one of a 'Series' of convertible notes issued to multiple investors (explains the separate ARM Holdings and Accrete convertible notes found in the same folder - those are OTHER investors in the same financing, not G42/Mozn). HIGH CONFIDENCE - document-verified. Entity renamed 'AAICO' -&gt; 'Applied AI' per user (2026-08-15): company later renamed; use 'Applied AI' going forward. Source folder is still named 'AAICO (desktop)'.</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BeyondLimits-EQ-2020</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>Beyond Limits</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MOZN Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>80000000</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2020-01-21</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Beyond Limits\2. Transaction Closure Documents\Beyond Limits - Investment Summary.docx</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>AI-extracted from Investment Summary + Note Purchase Agreement - Series C Preferred Stock tranche. HIGH CONFIDENCE.</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cerebras-SeriesF-2021</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>Cerebras</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Mozn Holding RSC Limited</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>39999983.36</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2021-10-19</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Cerebras\2. Investment $40m Oct 21\2. Transaction Documents\Cerebras - investment summary (6).docx</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>AI-extracted from Investment Summary: Series F Preferred, 1,441,711 shares, $39,999,983.36 paid 19 Oct 2021. HIGH CONFIDENCE. USER-CONFIRMED (2026-08-15) and now DOCUMENT-VERIFIED: after this initial round, G42 exercised Warrant 1 and Warrant 2 for Class N Common Stock (see Cerebras-Warrant1-2026 and Cerebras-Warrant2-2026 rows), bringing total share count to ~4.96M shares (~5M), matching user's account precisely. RESOLVED - no further follow-up needed for this round.</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DriveNets-EQ-2022</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>DriveNets</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>G42 SKY13 TECHNOLOGY PROJECTS RSC LTD</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2022-03-23</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PartiallyExited</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2025-03-14</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\DriveNets\1.1 Transaction docs Mar 2022\IAF, AoA, IRA\DriveNets - AT&amp;T Investment - Investment Summary - 29.07.2025.docx</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>CONFIRMED from Investment Approval Form (14 Mar 2022): $300M total = $200M primary + $100m secondary (buying from existing shareholders/employees), via Group 42 Holding Ltd's subsidiary G42 SKY13 TECHNOLOGY PROJECTS RSC LTD, structured as a fund with a G42 entity as LP and a Mozn entity as GP. Warrant: 101,215,211 Ordinary Shares (matches Investment Summary). HIGH CONFIDENCE - document-verified. NOTE: the 2025 AT&amp;T Investment Summary refers to the holder as 'D2 Investments RSC Ltd' - likely the same vehicle renamed/restructured since 2022, but not confirmed - flag if precision on entity continuity matters. SEPARATELY: there is a DRAFT Series D round (folder '1.2 Transaction Docs Mar 2026, Series D', pre-money valuation $8bn) with all investment amount fields still blank placeholders as of the draft - not yet a confirmed investment, not added as a row. The 2025 AT&amp;T secondary distribution (~$84.8M received by D2) is also still NOT booked as a cashflow row - needs adding when full details are available.</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>eSpace-EQ-2022</t>
+        </is>
+      </c>
       <c r="B6" t="inlineStr">
         <is>
           <t>e-space</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Smart InteractionS Holding SPV RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Convertible</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2022-11-27</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\e-space\2023.09.25 B1 and B2 Purchase and Sale Agreement.pdf</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>CONFIRMED from executed SAFE (Simple Agreement for Future Equity): Purchase Amount $15,000,000 exactly, investor Smart InteractionS Holding SPV RSC Ltd, Valuation Cap $675-700M. This resolves the earlier date mismatch - the SAFE (not the later PSA) is the actual close_date-relevant document, consistent with the 2022-11-27 tracker deployment. HIGH CONFIDENCE - document-verified, no longer a tracker fallback. The SAFE later converted into Class B-2 Preferred Stock per the Sep-2023 Purchase and Sale Agreement (see SAFE waiver documents dated Nov 2023). NOTE: the share certificate found is issued to 'Constellation Investments RSC SPV Ltd', a DIFFERENT name than the original SAFE investor - likely the same vehicle renamed, but not confirmed - flag if entity continuity matters.</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Endless-SeriesA-2021</t>
+        </is>
+      </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>Endless (Matt Dalio) and E-line</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2021-09-30</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Endless (Matt Dalio) and E-line\2. Series A Purchase Agreement Aug 21\20210907 Endless Studios Series A Summary Term Sheet(245805.1).pdf</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>AI-extracted from Term Sheet + Exhibit A cap table: G-42 Entity invested exactly $3,000,000 for 3,000,000 Preferred Class A Units (term sheet allowed a $3-7M range, but the actual pro forma cap table confirms $3M was the amount used), pre-money valuation $25M, closing 30 Sep 2021. HIGH CONFIDENCE on amount. fund_vehicle_id NOT explicitly named as a specific G42 SPV in this term sheet - needs the signed Purchase Agreement to confirm. Note: E-line Ventures LLC (tracker) shares this same folder/deal per earlier reconciliation.</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EsyaSoft-NOTE-2020</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>EsyaSoft</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MOZN Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Convertible</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2020-09-01</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\EsyaSoft\Esyasoft - Investment Summary.docx</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>AI-extracted from Investment Summary: $2.5M convertible note, 10% interest, 2yr term, converts to 21% fully diluted equity. HIGH CONFIDENCE.</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Flyr-SeriesB-2020</t>
+        </is>
+      </c>
       <c r="B9" t="inlineStr">
         <is>
           <t>Flyr</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MOZN Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2020-03-25</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Flyr\3. Monitoring\FlyR - Investment Summary.docx</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>AI-extracted: $5M cash for B-1 Prefs + $5M convertible note converted to B-2 Prefs = $10M total. HIGH CONFIDENCE.</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GlassEarth-NOTE-2019</t>
+        </is>
+      </c>
       <c r="B10" t="inlineStr">
         <is>
           <t>Glass Earth</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>G42 Investments RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Debt</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2019-06-19</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Glass Earth\Glass Earth - Promissory Note.jpg</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>AI-extracted via OCR (image scan): Promissory Note, $8,000,000 principal, dated 19 June 2019. Debtor: Sustainable Development Resources LLC (sole shareholder of Glass Earth Holdings LLC). Holder: G42 Investments RSC Ltd. Repayment date 21 June 2020, 12% penalty interest if late. HIGH CONFIDENCE on terms. USER-CONFIRMED (2026-08-15): the note DEFAULTED - the debtor took the money and disappeared; this is a complete write-off/loss, not a repayment. lifecycle_state = Exited, fully written off to $0.</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Heygears-EQ-2019</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>Heygears</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MOZN Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2019-09-30</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Heygears\1. Due Diligence Documents\Heygears - Investment Summary.docx</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>AI-extracted from Investment Summary: $60M for RMB4,753,356.29 registered capital, Equity Subscription Agreement 30 Sep 2019. HIGH CONFIDENCE. NOTE: folder '4.3 New round Jun 2026' contains THIRD-PARTY term sheets (Guangzhou Industrial Investment, Zhangjiagang Mingyi Lingxing, Shanghai Wofu) raising a NEW Series C round from OTHER investors - these are NOT G42 investments and were excluded from this row.</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>InstaDeep-EQ-2021</t>
+        </is>
+      </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>InstaDeep</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>5023720</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2021-12-20</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2023-10-25</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\InstaDeep\1. Due Diligence\AIC - InstaDeep Signed Term Sheet 2021.09.10.pdf</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>RECONCILED (user 2026-08-15): the tracker cashflow ($5,023,720 USD, 2021-12-20) reflects what Treasury actually transferred - this is the authoritative cash movement per our source-of-truth policy (Treasury owns cashflow truth). The signed Subscription Agreement denominates the share subscription in GBP (33,267 Class B Shares for GBP 3,679,995.54) - this is the contractual share-price basis, not necessarily the wire currency. Both figures are consistent (~1.365 GBP/USD implied rate). Recording USD $5,023,720 as initial_commitment_amount per Treasury's actual transfer; GBP 3,679,995.54 retained here for share-price/ownership traceability. fund_vehicle_id still shown only as '[G42]' bracket placeholder in the schedule - exact entity name unconfirmed.</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Inveniam-SAR-2024</t>
+        </is>
+      </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>Inveniam</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Expansion Project Technologies Holding 10 SPV RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Convertible</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>100032722.58</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2024-11-15</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Inveniam\6. Inveniam DD + Secondaries + Mantra Nov 2025\4. Dealdocs\9. Acies Investments Fund\CEF - Acies LPA SA and Side Letter.pdf</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FULLY CONFIRMED via two executed legal documents. (1) Original Token Purchase Agreement (15 Jun 2024): Mozn Holding Limited agreed to make a $100M investment in Inveniam Capital Partners, Inc. as part of the WLD token arrangement. (2) Amendment and Novation Agreement (6 Nov 2024): G42 Capital Limited novated its rights/obligations under that agreement to Expansion Project Technologies Holding 10 SPV RSC Ltd (EPTH), explicitly due to 'the prevailing market price of Worldcoin Tokens' prompting an alternative structure. (3) Convertible Stock Appreciation Rights Instrument (Grant Date 15 Nov 2024): EPTH granted 13,481,499 SARs over Inveniam Class D Preferred Stock at an exercise price of $7.42/SAR = $100,032,722.58 total notional value, equating to 20% of Inveniam's outstanding value at grant. Not yet exercised/converted. HIGH CONFIDENCE - fully document-verified chain, no longer relying on user recollection alone. Linked to TFH's $100M WLD-token distribution (TRK-CF-EQ-0049, tagged Non-Cash - Asset Exchange, ref 'WLD-Inveniam-SAR-Swap-2024') as the offsetting non-cash leg - this $100M cost basis was funded via token exchange, not fresh cash.</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Jysan-EQ-2021</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>Jysan Technologies</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>QAZ42 Investment SPV RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2021-04-06</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Jysan Technologies\2. Transaction Documents\1. Final Execution Documents\1. Jysan - Investment Summary.pdf</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>AI-extracted: $20M for 7,959,497 A Ordinary Shares (3%), Subscription Agreement 6 Apr 2021. HIGH CONFIDENCE.</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LifeBio-SeriesD-2024</t>
+        </is>
+      </c>
       <c r="B15" t="inlineStr">
         <is>
           <t>Life Biosciences</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Expansion Project Technologies Holding 7 SPV RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>40947395.44</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2024-10-28</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Life Biosciences\4.1 CFIUS related\Ex. B - Term Sheet(37056247_1).pdf</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>CONFIRMED from the actual FINAL executed Series D Purchase Agreement + its Disclosure Schedule (folder '4. 28 Oct 24'): Expansion Project Technologies Holding 7 SPV RSC Ltd (the 'Initial Purchaser') paid $19,999,998.17 cash for 6,925,351 Series D shares, plus a $20,947,397.27 Convertible Promissory Note converting into 7,253,404 further shares = $40,947,395.44 total. HIGH CONFIDENCE - document-verified, no longer based on a non-binding draft term sheet. close_date set to 28 Oct 2024 per the final docs folder.</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LiquidAI-SeriesA-2024</t>
+        </is>
+      </c>
       <c r="B16" t="inlineStr">
         <is>
           <t>Liquid AI</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Expansion Project Technologies Holding 11 SPV RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>66599843.43</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2024-12-23</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Liquid AI\1. Transaction Docs\Liquid AI - Executed Docs (G42) Nov 25\Liquid AI Inc. - Series A - G42 Side Letter [EXECUTED].pdf</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>AI-extracted from executed Side Letter: Initial G42 Closing $19,999,882.40 cash (165,082 shares) + Second G42 Closing $46,599,961.03 deemed consideration (384,643 shares, satisfied via compute cluster procurement, not cash) = $66,599,843.43 total Series A Preferred. HIGH CONFIDENCE on terms; note second tranche was non-cash (compute credit), worth flagging distinctly if precision matters.</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MenaMobile-SeriesB-2019</t>
+        </is>
+      </c>
       <c r="B17" t="inlineStr">
         <is>
           <t>MenaMobile</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MOZN Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2019-07-29</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\MenaMobile\1. Due Diligence Documents\Mena Mobile - Investment Summary.docx</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>AI-extracted: $8M for 21,419,829 Series B Preferred Shares, Agreement dated 29 Jul 2019. HIGH CONFIDENCE.</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Neuralink-SeriesE-2025</t>
+        </is>
+      </c>
       <c r="B18" t="inlineStr">
         <is>
           <t>Neuralink (Project Cortex)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Expansion Project Technologies Holding 12 SPV RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>49999999.5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Neuralink (Project Cortex)\Transaction Documents\Neuralink Investment Summary .docx</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>AI-extracted: 990,099 Series E Preferred shares @ $50.50/share = $49,999,999.50. Side Letter/IRA dated 30 May 2025; funding due by 4 June 2025 per Payment Direction Letter. HIGH CONFIDENCE.</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ONT-EQ-2020-Tranche1</t>
+        </is>
+      </c>
       <c r="B19" t="inlineStr">
         <is>
           <t>ONT</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>G42 AI Investments Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2020-05-19</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\ONT\2. Transaction Closure Documents\Oxford Nanopore - Investment Summary (Sep 2020) 4814-2336-4042 2.docx</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>AI-extracted: $50M paid 19 May 2020 for 763,884 Ordinary Shares. HIGH CONFIDENCE. RESOLVED (2026-08-15): found 'ONT Pre-Emption Rights' internal analysis (31 Mar 2021 folder) which independently cross-validates ALL prior tranches in USD terms (aggregate $130.3M / 2,101,050 shares by Aug-2020, matching the GBP figures previously recorded) AND explains the 115,356-share mystery: it was a separate Pre-IPO Pre-Emption Rights purchase on 30-Mar-2021 for $11.1M/GBP8.1M (see ONT-PreIPO-PreEmption-2021 row) - NOT the original 'Stage 2' ($30M Oxford + $26.875M JVCo) described in the 2020 Investment Summary. The original Stage 2 tranches remain UNCONFIRMED/UNRESOLVED - separate open question, not answered by this document. ONT listed on the London Stock Exchange (IPO ~Sep 2021); post-IPO substantial shareholder notifications (TR-1) are public but have not been checked yet. NEEDS FOLLOW-UP DOCUMENT for the original Stage 2 tranches. PUBLIC DISCLOSURE CHECKED (2026-08-15): ONT is LSE-listed; confirmed that TR-1 major shareholding notifications and the Annual Report's substantial-shareholdings table are publicly available (via nanoporetech.com/about/investors/regulatory-news, RNS/Investegate, or the LSE website), which would show G42's current stake and could confirm whether the original Stage 2 tranches occurred. Did not locate a specific G42 TR-1 filing yet - would require searching individual RNS announcements or the Annual Report for G42/Group 42's name. Left open per user's direction to move to next steps rather than continue searching now. USER-CONFIRMED (2026-08-15): the sub-1x TVPI is a REAL loss, not a data/valuation error. Value spiked substantially during COVID (large gains realized/marked then) and has declined substantially since. Direction of the return is correct; the original Stage 2 tranche question remains open only for precision on the exact invested/share-count figures, not because the loss itself is in doubt.</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SchoolHack-EQ-2024</t>
+        </is>
+      </c>
       <c r="B20" t="inlineStr">
         <is>
           <t>School Hack</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Core42 Investments 1 SPV RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2024-01-31</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\School Hack\Seed  - Mar 2024\9f. School Hack - Subscription Agreement - Updated Version 17012024[2].pdf</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>CONFIRMED from the actual Subscription Agreement, Clause 3.1: Core42 Investments 1 SPV RSC LTD subscribed 25,000 Preferred Shares for USD $2,500,000 - exact match to tracker figure. HIGH CONFIDENCE - document-verified, no longer a tracker fallback.</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TFH-SeriesC-2023</t>
+        </is>
+      </c>
       <c r="B21" t="inlineStr">
         <is>
           <t>TFH - Worldcoin</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2023-04-30</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\TFH - Worldcoin\1. DD Docs, IAF &amp; Closing Docs\2. Investment Note - Worldcoin\IC - Note\Investment summary note - Worldcoin - Apr-23.pdf</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>AI-extracted from Investment Summary Note (Apr 2023) + Term Sheet (3 Mar 2023): G42 allocation USD 30m in Series C Preferred + Token Warrants, Tools for Humanity Corporation (Worldcoin legal entity), post-money $2.4bn. HIGH CONFIDENCE on amount. fund_vehicle_id NOT explicitly named - needs the actual SPA. RESOLVED (user 2026-08-15): WLD tokens received were exchanged for ~$100M SAR in Inveniam - see Inveniam-SAR-TBD row. WLD token holding itself remains a separate line (already sold off per earlier note). ACCOUNTING TREATMENT AGREED (2026-08-15): the $100M WLD-token exchange (14 Nov 2024, cashflow TRK-CF-EQ-0049) is tagged 'Non-Cash - Asset Exchange' in Tracker_Extract_Reconciled (ref 'WLD-Inveniam-SAR-Swap-2024'). At the POSITION level this stays as-is (a real, legitimate ~6.66x distribution/gain on the WLD token holding - user confirmed a gain was booked on the WLD tokens). It should be EXCLUDED from any future PORTFOLIO-LEVEL aggregate cash paid-in/distributed/IRR calculation, since no actual cash left or entered the fund - it funded Inveniam's SAR directly. Per-position TVPI/MOIC for both TFH and Inveniam are correct as calculated; only a future aggregate rollup needs to filter this out.</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Verses-Debenture-2024</t>
+        </is>
+      </c>
       <c r="B22" t="inlineStr">
         <is>
           <t>Verses (Project Bayes)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Expansion Project Technologies Holding 9 SPV RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Convertible</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>13780000</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2024-06-20</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Verses (Project Bayes)\1. Letter of Intent\1. 09 Jan 24\Term Sheet for Convertible Debenture.docx</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>AI-extracted from EXECUTED Subscription Agreement: 13,780 Units @ CAD$1,000 = CAD$13,780,000 unsecured convertible debentures + warrants, 10% interest, 24-month maturity. HIGH CONFIDENCE (executed doc, not a draft).</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>VTVT-EQ-2022</t>
+        </is>
+      </c>
       <c r="B23" t="inlineStr">
         <is>
           <t>VTVT - vTv Therapeutics</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>G42 Health Care AI Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2022-02-18</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\VTVT - vTv Therapeutics\Transaction Docs\Term Sheet-vtv.pdf</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>AI-extracted via OCR (scanned PDF): Non-binding Term Sheet - G42 Health Care AI Holding RSC Ltd to acquire 10% of vTv Therapeutics Inc. common stock for $25M ($12.5M cash at closing + $12.5M secured note due in 1 year). A separate $20M milestone payment (in equity, upon FDA approval, funded via R&amp;D expenditure not cash) is NOT included in this amount. MEDIUM CONFIDENCE: this is a NON-BINDING draft term sheet, not a signed closing document - needs the actual signed agreement to confirm final terms. close_date is the folder date (18 Feb 22), not a date stated in the document itself.</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Xfusion-EQ-2022</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>X-fusion</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>493500956.2</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2022-01-13</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2023-10-25</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>TRACKER ONLY - no source document on file; figures derived from monthly tracker cashflow/NAV data (2 cashflow rows, 1 valuation rows)</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>HonorDevice-EQ-2022</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Honor Device Co Ltd</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>800000000</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2022-07-27</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2023-10-25</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>TRACKER ONLY - no source document on file; figures derived from monthly tracker cashflow/NAV data (4 cashflow rows, 1 valuation rows)</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Jollychic-EQ-2019</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Jollychic Holding Limited</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>65000000</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2019-01-05</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2019-09-16</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>TRACKER ONLY - no source document on file; figures derived from monthly tracker cashflow/NAV data (3 cashflow rows, 1 valuation rows)</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BeyondLimits-DEBT-2020</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Beyond Limits</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MOZN Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Convertible</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2020-01-21</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>AI-extracted: $20M convertible note @ 6% p.a., converts to C Prefs. HIGH CONFIDENCE.</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ONT-EQ-2020-PreEmptive</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ONT</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>G42 AI Investments Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>61632106</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2020-06-24</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>AI-extracted: 3 pre-emptive Oxford Ordinary Share payments - GBP21,029,625 (paid 24 Jun 2020), GBP14,386,480 (paid 3 Jul 2020), GBP26,216,001 (paid Aug 2020) = GBP61,632,106 total, cumulative shareholding reaching 2,101,050 Ordinary Shares - independently confirmed by a Deloitte letter dated 16 Mar 2021 re: 31 Dec 2020 status. HIGH CONFIDENCE. close_date set to the first of the 3 payments.</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ONT-JVCo-2020</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ONT</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>G42 AI Investments Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>3125000</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2020-04-29</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>AI-extracted: $3.125M for B Ordinary Shares in JVCo (the separate G42/Oxford joint venture entity, NOT Oxford Nanopore itself) - marked 'Paid' in the source document but no specific payment date given; close_date approximated to the Framework Agreement date (29 Apr 2020). MEDIUM CONFIDENCE on date only.</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Cerebras-Warrant1-2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Cerebras</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Core42 Holding US LLC</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>18575.16</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>AI-extracted from executed Warrant 1 + Notice of Exercise: 1,857,516 shares of Class N Common Stock at $0.01/share = $18,575.16 total exercise cost. Warrant executed 30 Dec 2025, exercised 5 Jan 2026 by Core42 Holding US LLC. Matches tracker cashflow exactly. HIGH CONFIDENCE - document-verified. Note: nominal cost reflects the exercise price only, not the fair value of shares received.</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cerebras-Warrant2-2026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Cerebras</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Expansion Project Technologies Holding 8 SPV RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>16559.75</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>AI-extracted from Warrant 2 (2026.04.10 Final Clean): 1,655,975 shares of Class N Common Stock at $0.01/share = $16,559.75. Vests on execution of a Statement of Work (Condor Galaxies 14/15/16 HPC clusters) by 13 Apr 2026, expires 15 Apr 2026. Holder: Expansion Project Technologies Holding 8 SPV RSC Ltd. Matches tracker cashflow ($16,559.75, dated 2026-04-17) exactly. HIGH CONFIDENCE - document-verified. Note: nominal cost reflects the exercise price only, not fair value received.</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ONT-PreIPO-PreEmption-2021</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ONT</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>G42 AI Investments Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>11100000</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2021-03-30</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>AI-extracted from 'ONT Pre-Emption Rights' internal analysis (31 Mar 2021 folder): Pre-IPO Pre-Emption Rights offering, 115,356 shares at GBP70.00/$96.60 per share = approx. $11.1M / GBP8.1M (document gives only rounded figures, not exact cents). This brought G42's total to 2,216,406 shares (6.14-6.46% ownership) ahead of the IPO. HIGH CONFIDENCE on mechanism and approximate amount.</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NewSpace-ICEYE-2020</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1. New Space Capital Fund</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>G42 Investments AI Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>FundInterest</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>19015957.27</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2020-09-03</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>CONFIRMED from signed Side Letter + Drawdown 1 Notice (3 Sep 2020): New Space Capital Fund I is an SPV-style vehicle with a separate 'Sub-Fund' per deal - this is the ICEYE Oy sub-fund only (1,591,574 Series C preferred shares, 6.1% of ICEYE, EUR18,798,671.27 + fees = EUR19,015,957.27 total commitment, fully drawn at this single Drawdown 1). HIGH CONFIDENCE for THIS sub-fund. NEEDS FOLLOW-UP DOCUMENT: 20 total drawdown notices exist through 2025 in this fund's folder, indicating MULTIPLE additional sub-fund deals beyond ICEYE (tracker shows ~$36M total paid-in across 23 cashflow rows, far more than this one EUR19M sub-fund) - not yet individually identified/recorded.</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sinovation-LP-2020</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2. Sinovation Disrupt Fund</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>G42 Investments AI Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>FundInterest</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2020-11-18</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>CONFIRMED from Partners Capital Account Statement (as at 31 Dec 2020): G42 Investments AI Holding RSC Ltd, Total Capital Commitment $50,000,000, Partnership Percentage 36.63%. close_date approximated to the first tracker capital call (18 Nov 2020) - exact LPA/Subscription Agreement signing date not yet located. HIGH CONFIDENCE on commitment amount and investor entity.</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NorthSummit-LP-2019</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2. North Summit Capital Fund</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Galbot Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FundInterest</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2019-06-18</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>CONFIRMED from Capital Call Notice #1 (21 Jun 2019): Total Capital Commitment USD 300,000,000 (100%), Limited Partner is 'Galbot Holding RSC Ltd' (a G42 SPV) per the Subscription Agreement and A&amp;R LPA. First drawdown was only 1% ($3M). close_date approximated to 18 Jun 2019 (fee period start date referenced in the notice). HIGH CONFIDENCE on commitment amount and vehicle name. NOTE: folder contains a '3. Liquidation FY25' subfolder - possible wind-down in progress, not yet investigated.</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Acies-LP-2021</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>3. ACIES</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>G42 Investments AI Holding RSC Ltd</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FundInterest</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2021-11-15</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>CONFIRMED from executed CEF (15 Nov 2021) + Anchor MOU Terms: LP commitment of the lesser of 50% of aggregate LP commitments or $50M in Acies Ventures Fund I, L.P. (target fund size $150M), via G42 Investments AI Holding RSC Ltd. ADDITIONAL RIGHT not reflected in this $ figure: G42/Mozn is also an economic assignee entitled to 9.9% of the GP's carried interest - a separate, non-capital economic interest not captured as a register row. HIGH CONFIDENCE on the $50M LP commitment.</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>MGX-I-LP-2024</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>4. MGX</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>GX Investments Ltd</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>FundInterest</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1189553910</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2024-05-08</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>CONFIRMED from Capital Account Statement (as of 31 Dec 2024): MGX I LP, Investor GX Investments Ltd, Total Commitment $1,189,553,910, Paid-in Capital $116,097,286 (8.08% ownership of fund). close_date uses the statement's 'Opening Balance Date' (08 May 2024) as a proxy - the actual original LPA/subscription signing date has not been located. HIGH CONFIDENCE on commitment figure.</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>MGX-I-StrategicCoInvest-2024</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>4. MGX</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>GX Investments Ltd</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>FundInterest</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>775000000</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2024-10-01</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>CONFIRMED from Capital Account Statement (as of 31 Dec 2024): MGX I Strategic Co-Invest LP, Investor GX Investments Ltd, Total Commitment $775,000,000, Paid-in Capital $249,999,999 (50.00% ownership). close_date uses the statement's 'Opening Balance Date' (01 Oct 2024) as a proxy. HIGH CONFIDENCE on commitment figure.</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MGX-I-DenaliHolding-2024</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>4. MGX</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>GX Investments US LLC</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>FundInterest</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>27672749</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2024-10-01</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>UPDATED 2026-08-15 from MGX I Denali Holding LP - Capital Account Statement - Q3 2025_GX Investments US LLC.pdf (primary document, Since Inception column): GX Investments US LLC's allocation - Total Commitment $27,672,749, fully called (Contributions - Since Inception = $27,672,749), Ending NAV (carrying value) $41,594,050 as of 30-Sep-2025. Supersedes the earlier Dec-2024 CAS figure ($10,446,090) - Denali's commitment was increased/topped-up between Dec 2024 and Q3 2025. HIGH CONFIDENCE (primary capital account statement, both commitment and carrying value).</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>MGX-GroupHolding1-GP-2024</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>4. MGX</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MGX Group Holding 1 Ltd (GP)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>FundInterest</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2024-05-08</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Tracker: dedicated 'MGX' tab (Source: Capital Account Statement Q3'25) + NAV tab, Jul'26 v2.0</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>CONFIRMED per user (2026-08-15): G42 funded MGX's GP costs as a 3rd distinct MGX vehicle (alongside the fund LP MGX I LP and the co-invest vehicles MGX I Strategic Co-Invest LP / MGX I Denali Holding LP) - a real economic position, not a wrapper/pass-through to exclude. Amount ($25,000,000, fully funded, static TVPI 1.0x across all tracker periods) sourced from the tracker's dedicated 'MGX' tab (labeled 'Source: Capital Account Statement Q3 25') and the NAV tab's 'MGX Group Holding 1 Ltd (GP)' carrying value row (also $25,000,000, as of 31-Jul-2026 NAV date). MEDIUM CONFIDENCE: no independent legal/subscription document for this specific GP-level stake was located in the MGX documents folder (searched '4. MGX' folder and investments-root-wide for 'Group Holding'/'GP Interest'/'Sponsor' filenames - none found beyond the fund-level audited financial statements, which confirm 'MGX GP 1 RSC Ltd' as MGX I LP's General Partner but do not separately disclose this stake). Treated as the same entity as the tracker's 'MGX HoldCo' cashflow-tab name (see Entity_Reconciliation) - both show exactly $25,000,000, one-time, fully called, no other MGX line item is unexplained at this amount.</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>NewSpace-GPCom-2023</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1. New Space Capital Fund</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>NewSpace Capital GP Com SCSp</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>FundInterest</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2020-09-13</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2023-03-21</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>NSC GP Com SCSp_LPA_21 March 2023.pdf; Restructuring Agreement 20221102_Execution version (002).pdf; G42 _ NewSpace - Legal summary(28008631_1).DOCX</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>CONFIRMED 2026-08-15 from 3 primary documents read in sequence: (1) 'G42 _ NewSpace - Legal summary (28008631_1).DOCX' - original 2020 commitment: G42 to acquire 167 Class C Units in 'NewSpace Capital Partners SCSp' (the carry/GP-economics vehicle sitting above the Fund's General Partner) for EUR 2,300,000, entitling G42 to 26.67% of 75% of carried interest on the ICEYE investment (and 11.11% of 75% on any other Sub-Fund investments). (2) 'Restructuring Agreement 20221102' - on 2 Nov 2022, following a new EUR 75,000,000 LP commitment from Archean Capital Partners (Class A Units) into the Fund, G42's Class C Units position (by then 171 units) in NewSpace Capital Partners SCSp was transformed into a new 'GP Commitment Vehicle' sitting between the Partnership and the Fund. (3) 'NSC GP Com SCSp_LPA_21 March 2023.pdf' - the governing LPA for this GP Commitment Vehicle, now named 'NewSpace Capital GP Com SCSp' - matches the tracker's 'New Space Capital GP Com SCSp' cashflow name exactly. Tracker shows $2.125M paid-in / $0.175M distributed against this original EUR 2,300,000 commitment - consistent (not fully called, some FX/timing variance). HIGH CONFIDENCE on economic substance and lineage; MEDIUM CONFIDENCE on exact close_date (used the Fund's own Drawdown 1 date, 2020-09-13, as a proxy since the original Partnership investment was contemporaneous with the Fund's first drawdown per the legal summary, but no exact signing date was found in that document).</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6317,4 +7862,84 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>entity_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>investment_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>gap_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ONT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ONT-EQ-2020-Tranche1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NEEDS FOLLOW-UP</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AI-extracted: $50M paid 19 May 2020 for 763,884 Ordinary Shares. HIGH CONFIDENCE. RESOLVED (2026-08-15): found 'ONT Pre-Emption Rights' internal analysis (31 Mar 2021 folder) which independently cross-validates ALL prior tranches in USD terms (aggregate $130.3M / 2,101,050 shares by Aug-2020, matching the GBP figures previously recorded) AND explains the 115,356-share mystery: it was a separate Pre-IPO Pre-Emption Rights purchase on 30-Mar-2021 for $11.1M/GBP8.1M (see ONT-PreIPO-PreEmption-2021 row) - NOT the original 'Stage 2' ($30M Oxford + $26.875M JVCo) described in the 2020 Investment Summary. The original Stage 2 tranches remain UNCONFIRMED/UNRESOLVED - separate open question, not answered by this document. ONT listed on the London Stock Exchange (IPO ~Sep 2021); post-IPO substantial shareholder notifications (TR-1) are public but have not been checked yet. NEEDS FOLLOW-UP DOCUMENT for the original Stage 2 tranches. PUBLIC DISCLOSURE CHECKED (2026-08-15): ONT is LSE-listed; confirmed that TR-1 major shareholding notifications and the Annual Report's substantial-shareholdings table are publicly available (via nanoporetech.com/about/investors/regulatory-news, RNS/Investegate, or the LSE website), which would show G42's current stake and could confirm whether the original Stage 2 tranches occurred. Did not locate a specific G42 TR-1 filing yet - would require searching individual RNS announcements or the Annual Report for G42/Group 42's name. Left open per user's direction to move to next steps rather than continue searching now. USER-CONFIRMED (2026-08-15): the sub-1x TVPI is a REAL loss, not a data/valuation error. Value spiked substantially during COVID (large gains realized/marked then) and has declined substantially since. Direction of the return is correct; the original Stage 2 tranche question remains open only for precision on the exact invested/share-count figures, not because the loss itself is in doubt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1. New Space Capital Fund</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NewSpace-ICEYE-2020</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NEEDS FOLLOW-UP</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CONFIRMED from signed Side Letter + Drawdown 1 Notice (3 Sep 2020): New Space Capital Fund I is an SPV-style vehicle with a separate 'Sub-Fund' per deal - this is the ICEYE Oy sub-fund only (1,591,574 Series C preferred shares, 6.1% of ICEYE, EUR18,798,671.27 + fees = EUR19,015,957.27 total commitment, fully drawn at this single Drawdown 1). HIGH CONFIDENCE for THIS sub-fund. NEEDS FOLLOW-UP DOCUMENT: 20 total drawdown notices exist through 2025 in this fund's folder, indicating MULTIPLE additional sub-fund deals beyond ICEYE (tracker shows ~$36M total paid-in across 23 cashflow rows, far more than this one EUR19M sub-fund) - not yet individually identified/recorded.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>